<commit_message>
stage Alpha v2.6.0 workbook import audit
</commit_message>
<xml_diff>
--- a/assets/source-archive/alpha-v260-xlsx-import/sources/法术卡列表.xlsx
+++ b/assets/source-archive/alpha-v260-xlsx-import/sources/法术卡列表.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Project\WizardCard-Design\Alpha 现有卡池\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACD0B4BB-E98F-413E-ADD6-FC4BF7B22FA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7315636F-2767-411D-B26A-D7370BCCA7D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25710" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="卡表" sheetId="1" r:id="rId1"/>
@@ -1181,7 +1181,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -1707,22 +1707,22 @@
     <tabColor rgb="FF1F4E79"/>
   </sheetPr>
   <dimension ref="A1:M203"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="6.28515625" customWidth="1"/>
-    <col min="2" max="2" width="10.28515625" customWidth="1"/>
-    <col min="3" max="3" width="8.28515625" customWidth="1"/>
-    <col min="4" max="4" width="19.28515625" customWidth="1"/>
-    <col min="5" max="5" width="7.28515625" customWidth="1"/>
-    <col min="6" max="6" width="6.28515625" customWidth="1"/>
-    <col min="7" max="8" width="16.28515625" customWidth="1"/>
-    <col min="9" max="10" width="10.28515625" customWidth="1"/>
-    <col min="11" max="11" width="94.42578125" customWidth="1"/>
-    <col min="12" max="12" width="15.28515625" customWidth="1"/>
-    <col min="13" max="13" width="9.28515625" customWidth="1"/>
+    <col min="1" max="1" width="6.26953125" customWidth="1"/>
+    <col min="2" max="2" width="10.26953125" customWidth="1"/>
+    <col min="3" max="3" width="8.26953125" customWidth="1"/>
+    <col min="4" max="4" width="19.26953125" customWidth="1"/>
+    <col min="5" max="5" width="7.26953125" customWidth="1"/>
+    <col min="6" max="6" width="6.26953125" customWidth="1"/>
+    <col min="7" max="8" width="16.26953125" customWidth="1"/>
+    <col min="9" max="10" width="10.26953125" customWidth="1"/>
+    <col min="11" max="11" width="94.453125" customWidth="1"/>
+    <col min="12" max="12" width="15.26953125" customWidth="1"/>
+    <col min="13" max="13" width="9.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="32.15" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1763,7 +1763,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="30" customHeight="1">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -1800,7 +1800,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="30" customHeight="1">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -1837,7 +1837,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="30" customHeight="1">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -1874,7 +1874,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="30" customHeight="1">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -1911,7 +1911,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="30" customHeight="1">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -1948,7 +1948,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="30" customHeight="1">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -1985,7 +1985,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" ht="30" customHeight="1">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -2022,7 +2022,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" ht="30" customHeight="1">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -2059,7 +2059,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" ht="30" customHeight="1">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -2096,7 +2096,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" ht="30" customHeight="1">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -2135,7 +2135,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" ht="30" customHeight="1">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -2172,7 +2172,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" ht="30" customHeight="1">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -2209,7 +2209,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" ht="30" customHeight="1">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -2248,7 +2248,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" ht="30" customHeight="1">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -2287,7 +2287,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" ht="30" customHeight="1">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -2326,7 +2326,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" ht="30" customHeight="1">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -2363,7 +2363,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" ht="30" customHeight="1">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -2402,7 +2402,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" ht="30" customHeight="1">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -2441,7 +2441,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" ht="30" customHeight="1">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -2478,7 +2478,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" ht="30" customHeight="1">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -2515,7 +2515,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" ht="30" customHeight="1">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -2552,7 +2552,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" ht="30" customHeight="1">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -2591,7 +2591,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" ht="30" customHeight="1">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -2630,7 +2630,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" ht="30" customHeight="1">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -2669,7 +2669,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" ht="30" customHeight="1">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -2706,7 +2706,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" ht="30" customHeight="1">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -2745,7 +2745,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="28" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" ht="30" customHeight="1">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -2784,7 +2784,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="29" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" ht="30" customHeight="1">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -2823,7 +2823,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="30" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" ht="30" customHeight="1">
       <c r="A30" s="3">
         <v>29</v>
       </c>
@@ -2860,7 +2860,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="31" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" ht="30" customHeight="1">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -2899,7 +2899,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="32" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" ht="30" customHeight="1">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -2938,7 +2938,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="33" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" ht="30" customHeight="1">
       <c r="A33" s="3">
         <v>32</v>
       </c>
@@ -2977,7 +2977,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="34" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" ht="30" customHeight="1">
       <c r="A34" s="3">
         <v>33</v>
       </c>
@@ -3016,7 +3016,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="35" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" ht="30" customHeight="1">
       <c r="A35" s="3">
         <v>34</v>
       </c>
@@ -3055,7 +3055,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="36" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" ht="30" customHeight="1">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -3092,7 +3092,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="37" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" ht="30" customHeight="1">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -3129,7 +3129,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="38" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" ht="30" customHeight="1">
       <c r="A38" s="3">
         <v>37</v>
       </c>
@@ -3168,7 +3168,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="39" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" ht="30" customHeight="1">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -3207,7 +3207,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="40" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:13" ht="30" customHeight="1">
       <c r="A40" s="3">
         <v>39</v>
       </c>
@@ -3246,7 +3246,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="41" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:13" ht="30" customHeight="1">
       <c r="A41" s="17"/>
       <c r="B41" s="17"/>
       <c r="C41" s="17"/>
@@ -3261,7 +3261,7 @@
       <c r="L41" s="17"/>
       <c r="M41" s="17"/>
     </row>
-    <row r="42" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:13" ht="30" customHeight="1">
       <c r="A42" s="3">
         <v>1</v>
       </c>
@@ -3298,7 +3298,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="43" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:13" ht="30" customHeight="1">
       <c r="A43" s="3">
         <v>2</v>
       </c>
@@ -3327,7 +3327,7 @@
         <v>0</v>
       </c>
       <c r="J43" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K43" s="7" t="s">
         <v>196</v>
@@ -3337,7 +3337,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="44" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:13" ht="30" customHeight="1">
       <c r="A44" s="3">
         <v>3</v>
       </c>
@@ -3374,7 +3374,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="45" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:13" ht="30" customHeight="1">
       <c r="A45" s="3">
         <v>4</v>
       </c>
@@ -3413,7 +3413,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="46" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:13" ht="30" customHeight="1">
       <c r="A46" s="3">
         <v>5</v>
       </c>
@@ -3450,7 +3450,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="47" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:13" ht="30" customHeight="1">
       <c r="A47" s="3">
         <v>6</v>
       </c>
@@ -3487,7 +3487,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="48" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:13" ht="30" customHeight="1">
       <c r="A48" s="3">
         <v>7</v>
       </c>
@@ -3524,7 +3524,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="49" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:13" ht="30" customHeight="1">
       <c r="A49" s="3">
         <v>8</v>
       </c>
@@ -3561,7 +3561,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="50" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:13" ht="30" customHeight="1">
       <c r="A50" s="3">
         <v>9</v>
       </c>
@@ -3600,7 +3600,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="51" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:13" ht="30" customHeight="1">
       <c r="A51" s="3">
         <v>10</v>
       </c>
@@ -3639,7 +3639,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="52" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:13" ht="30" customHeight="1">
       <c r="A52" s="3">
         <v>11</v>
       </c>
@@ -3678,7 +3678,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="53" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:13" ht="30" customHeight="1">
       <c r="A53" s="3">
         <v>12</v>
       </c>
@@ -3717,7 +3717,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="54" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:13" ht="30" customHeight="1">
       <c r="A54" s="3">
         <v>13</v>
       </c>
@@ -3756,7 +3756,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="55" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:13" ht="30" customHeight="1">
       <c r="A55" s="3">
         <v>14</v>
       </c>
@@ -3795,7 +3795,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="56" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:13" ht="30" customHeight="1">
       <c r="A56" s="3">
         <v>15</v>
       </c>
@@ -3834,7 +3834,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="57" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:13" ht="30" customHeight="1">
       <c r="A57" s="3">
         <v>16</v>
       </c>
@@ -3873,7 +3873,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="58" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:13" ht="30" customHeight="1">
       <c r="A58" s="3">
         <v>17</v>
       </c>
@@ -3910,7 +3910,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="59" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:13" ht="30" customHeight="1">
       <c r="A59" s="3">
         <v>18</v>
       </c>
@@ -3947,7 +3947,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="60" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:13" ht="30" customHeight="1">
       <c r="A60" s="3">
         <v>19</v>
       </c>
@@ -3986,7 +3986,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="61" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:13" ht="30" customHeight="1">
       <c r="A61" s="3">
         <v>20</v>
       </c>
@@ -4025,7 +4025,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="62" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:13" ht="30" customHeight="1">
       <c r="A62" s="3">
         <v>21</v>
       </c>
@@ -4064,7 +4064,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="63" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:13" ht="30" customHeight="1">
       <c r="A63" s="17"/>
       <c r="B63" s="17"/>
       <c r="C63" s="17"/>
@@ -4079,7 +4079,7 @@
       <c r="L63" s="17"/>
       <c r="M63" s="17"/>
     </row>
-    <row r="64" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:13" ht="30" customHeight="1">
       <c r="A64" s="3">
         <v>1</v>
       </c>
@@ -4118,7 +4118,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="65" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:13" ht="30" customHeight="1">
       <c r="A65" s="3">
         <v>2</v>
       </c>
@@ -4157,7 +4157,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="66" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:13" ht="30" customHeight="1">
       <c r="A66" s="3">
         <v>3</v>
       </c>
@@ -4194,7 +4194,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="67" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:13" ht="30" customHeight="1">
       <c r="A67" s="3">
         <v>4</v>
       </c>
@@ -4231,7 +4231,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="68" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:13" ht="30" customHeight="1">
       <c r="A68" s="3">
         <v>5</v>
       </c>
@@ -4268,7 +4268,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="69" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:13" ht="30" customHeight="1">
       <c r="A69" s="3">
         <v>6</v>
       </c>
@@ -4307,7 +4307,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="70" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:13" ht="30" customHeight="1">
       <c r="A70" s="3">
         <v>7</v>
       </c>
@@ -4346,7 +4346,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="71" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:13" ht="30" customHeight="1">
       <c r="A71" s="3">
         <v>8</v>
       </c>
@@ -4385,7 +4385,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="72" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:13" ht="30" customHeight="1">
       <c r="A72" s="3">
         <v>9</v>
       </c>
@@ -4422,7 +4422,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="73" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:13" ht="30" customHeight="1">
       <c r="A73" s="3">
         <v>10</v>
       </c>
@@ -4459,7 +4459,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="74" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:13" ht="30" customHeight="1">
       <c r="A74" s="3">
         <v>11</v>
       </c>
@@ -4498,7 +4498,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="75" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:13" ht="30" customHeight="1">
       <c r="A75" s="3">
         <v>12</v>
       </c>
@@ -4537,388 +4537,388 @@
         <v>378</v>
       </c>
     </row>
-    <row r="76" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:13" ht="15" customHeight="1">
       <c r="H76" s="10"/>
     </row>
-    <row r="77" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:13" ht="15" customHeight="1">
       <c r="H77" s="10"/>
     </row>
-    <row r="78" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:13" ht="15" customHeight="1">
       <c r="H78" s="10"/>
     </row>
-    <row r="79" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:13" ht="15" customHeight="1">
       <c r="H79" s="10"/>
     </row>
-    <row r="80" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:13" ht="15" customHeight="1">
       <c r="H80" s="10"/>
     </row>
-    <row r="81" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="8:8" ht="15" customHeight="1">
       <c r="H81" s="10"/>
     </row>
-    <row r="82" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="8:8" ht="15" customHeight="1">
       <c r="H82" s="10"/>
     </row>
-    <row r="83" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="8:8" ht="15" customHeight="1">
       <c r="H83" s="10"/>
     </row>
-    <row r="84" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="8:8" ht="15" customHeight="1">
       <c r="H84" s="10"/>
     </row>
-    <row r="85" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="8:8" ht="15" customHeight="1">
       <c r="H85" s="10"/>
     </row>
-    <row r="86" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="8:8" ht="15" customHeight="1">
       <c r="H86" s="10"/>
     </row>
-    <row r="87" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="8:8" ht="15" customHeight="1">
       <c r="H87" s="10"/>
     </row>
-    <row r="88" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="8:8" ht="15" customHeight="1">
       <c r="H88" s="10"/>
     </row>
-    <row r="89" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="8:8" ht="15" customHeight="1">
       <c r="H89" s="10"/>
     </row>
-    <row r="90" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="8:8" ht="15" customHeight="1">
       <c r="H90" s="10"/>
     </row>
-    <row r="91" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="8:8" ht="15" customHeight="1">
       <c r="H91" s="10"/>
     </row>
-    <row r="92" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="8:8" ht="15" customHeight="1">
       <c r="H92" s="10"/>
     </row>
-    <row r="93" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="8:8" ht="15" customHeight="1">
       <c r="H93" s="10"/>
     </row>
-    <row r="94" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="8:8" ht="15" customHeight="1">
       <c r="H94" s="10"/>
     </row>
-    <row r="95" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="8:8" ht="15" customHeight="1">
       <c r="H95" s="10"/>
     </row>
-    <row r="96" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="8:8" ht="15" customHeight="1">
       <c r="H96" s="10"/>
     </row>
-    <row r="97" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="8:8" ht="15" customHeight="1">
       <c r="H97" s="10"/>
     </row>
-    <row r="98" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="8:8" ht="15" customHeight="1">
       <c r="H98" s="10"/>
     </row>
-    <row r="99" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="8:8" ht="15" customHeight="1">
       <c r="H99" s="10"/>
     </row>
-    <row r="100" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="8:8" ht="15" customHeight="1">
       <c r="H100" s="10"/>
     </row>
-    <row r="101" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="8:8" ht="15" customHeight="1">
       <c r="H101" s="10"/>
     </row>
-    <row r="102" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="8:8" ht="15" customHeight="1">
       <c r="H102" s="10"/>
     </row>
-    <row r="103" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="8:8" ht="15" customHeight="1">
       <c r="H103" s="10"/>
     </row>
-    <row r="104" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="8:8" ht="15" customHeight="1">
       <c r="H104" s="10"/>
     </row>
-    <row r="105" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="8:8" ht="15" customHeight="1">
       <c r="H105" s="10"/>
     </row>
-    <row r="106" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="8:8" ht="15" customHeight="1">
       <c r="H106" s="10"/>
     </row>
-    <row r="107" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="8:8" ht="15" customHeight="1">
       <c r="H107" s="10"/>
     </row>
-    <row r="108" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="8:8" ht="15" customHeight="1">
       <c r="H108" s="10"/>
     </row>
-    <row r="109" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="8:8" ht="15" customHeight="1">
       <c r="H109" s="10"/>
     </row>
-    <row r="110" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="8:8" ht="15" customHeight="1">
       <c r="H110" s="10"/>
     </row>
-    <row r="111" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="8:8" ht="15" customHeight="1">
       <c r="H111" s="10"/>
     </row>
-    <row r="112" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="8:8" ht="15" customHeight="1">
       <c r="H112" s="10"/>
     </row>
-    <row r="113" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="8:8" ht="15" customHeight="1">
       <c r="H113" s="10"/>
     </row>
-    <row r="114" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="8:8" ht="15" customHeight="1">
       <c r="H114" s="10"/>
     </row>
-    <row r="115" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="8:8" ht="15" customHeight="1">
       <c r="H115" s="10"/>
     </row>
-    <row r="116" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="8:8" ht="15" customHeight="1">
       <c r="H116" s="10"/>
     </row>
-    <row r="117" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="8:8" ht="15" customHeight="1">
       <c r="H117" s="10"/>
     </row>
-    <row r="118" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="8:8" ht="15" customHeight="1">
       <c r="H118" s="10"/>
     </row>
-    <row r="119" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="8:8" ht="15" customHeight="1">
       <c r="H119" s="10"/>
     </row>
-    <row r="120" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="8:8" ht="15" customHeight="1">
       <c r="H120" s="10"/>
     </row>
-    <row r="121" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="8:8" ht="15" customHeight="1">
       <c r="H121" s="10"/>
     </row>
-    <row r="122" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="8:8" ht="15" customHeight="1">
       <c r="H122" s="10"/>
     </row>
-    <row r="123" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="8:8" ht="15" customHeight="1">
       <c r="H123" s="10"/>
     </row>
-    <row r="124" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="8:8" ht="15" customHeight="1">
       <c r="H124" s="10"/>
     </row>
-    <row r="125" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="8:8" ht="15" customHeight="1">
       <c r="H125" s="10"/>
     </row>
-    <row r="126" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="8:8" ht="15" customHeight="1">
       <c r="H126" s="10"/>
     </row>
-    <row r="127" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="8:8" ht="15" customHeight="1">
       <c r="H127" s="10"/>
     </row>
-    <row r="128" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="8:8" ht="15" customHeight="1">
       <c r="H128" s="10"/>
     </row>
-    <row r="129" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="8:8" ht="15" customHeight="1">
       <c r="H129" s="10"/>
     </row>
-    <row r="130" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="8:8" ht="15" customHeight="1">
       <c r="H130" s="10"/>
     </row>
-    <row r="131" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="8:8" ht="15" customHeight="1">
       <c r="H131" s="10"/>
     </row>
-    <row r="132" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="8:8" ht="15" customHeight="1">
       <c r="H132" s="10"/>
     </row>
-    <row r="133" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="8:8" ht="15" customHeight="1">
       <c r="H133" s="10"/>
     </row>
-    <row r="134" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="8:8" ht="15" customHeight="1">
       <c r="H134" s="10"/>
     </row>
-    <row r="135" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="8:8" ht="15" customHeight="1">
       <c r="H135" s="10"/>
     </row>
-    <row r="136" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="8:8" ht="15" customHeight="1">
       <c r="H136" s="10"/>
     </row>
-    <row r="137" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="8:8" ht="15" customHeight="1">
       <c r="H137" s="10"/>
     </row>
-    <row r="138" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="8:8" ht="15" customHeight="1">
       <c r="H138" s="10"/>
     </row>
-    <row r="139" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="8:8" ht="15" customHeight="1">
       <c r="H139" s="10"/>
     </row>
-    <row r="140" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="8:8" ht="15" customHeight="1">
       <c r="H140" s="10"/>
     </row>
-    <row r="141" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="8:8" ht="15" customHeight="1">
       <c r="H141" s="10"/>
     </row>
-    <row r="142" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="8:8" ht="15" customHeight="1">
       <c r="H142" s="10"/>
     </row>
-    <row r="143" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="8:8" ht="15" customHeight="1">
       <c r="H143" s="10"/>
     </row>
-    <row r="144" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="8:8" ht="15" customHeight="1">
       <c r="H144" s="10"/>
     </row>
-    <row r="145" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="8:8" ht="15" customHeight="1">
       <c r="H145" s="10"/>
     </row>
-    <row r="146" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="8:8" ht="15" customHeight="1">
       <c r="H146" s="10"/>
     </row>
-    <row r="147" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="8:8" ht="15" customHeight="1">
       <c r="H147" s="10"/>
     </row>
-    <row r="148" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="8:8" ht="15" customHeight="1">
       <c r="H148" s="10"/>
     </row>
-    <row r="149" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="8:8" ht="15" customHeight="1">
       <c r="H149" s="10"/>
     </row>
-    <row r="150" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="8:8" ht="15" customHeight="1">
       <c r="H150" s="10"/>
     </row>
-    <row r="151" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="8:8" ht="15" customHeight="1">
       <c r="H151" s="10"/>
     </row>
-    <row r="152" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="8:8" ht="15" customHeight="1">
       <c r="H152" s="10"/>
     </row>
-    <row r="153" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="8:8" ht="15" customHeight="1">
       <c r="H153" s="10"/>
     </row>
-    <row r="154" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="8:8" ht="15" customHeight="1">
       <c r="H154" s="10"/>
     </row>
-    <row r="155" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="8:8" ht="15" customHeight="1">
       <c r="H155" s="10"/>
     </row>
-    <row r="156" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="8:8" ht="15" customHeight="1">
       <c r="H156" s="10"/>
     </row>
-    <row r="157" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="8:8" ht="15" customHeight="1">
       <c r="H157" s="10"/>
     </row>
-    <row r="158" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="8:8" ht="15" customHeight="1">
       <c r="H158" s="10"/>
     </row>
-    <row r="159" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="8:8" ht="15" customHeight="1">
       <c r="H159" s="10"/>
     </row>
-    <row r="160" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="8:8" ht="15" customHeight="1">
       <c r="H160" s="10"/>
     </row>
-    <row r="161" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="8:8" ht="15" customHeight="1">
       <c r="H161" s="10"/>
     </row>
-    <row r="162" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="8:8" ht="15" customHeight="1">
       <c r="H162" s="10"/>
     </row>
-    <row r="163" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="8:8" ht="15" customHeight="1">
       <c r="H163" s="10"/>
     </row>
-    <row r="164" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="8:8" ht="15" customHeight="1">
       <c r="H164" s="10"/>
     </row>
-    <row r="165" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="8:8" ht="15" customHeight="1">
       <c r="H165" s="10"/>
     </row>
-    <row r="166" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="8:8" ht="15" customHeight="1">
       <c r="H166" s="10"/>
     </row>
-    <row r="167" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="8:8" ht="15" customHeight="1">
       <c r="H167" s="10"/>
     </row>
-    <row r="168" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="8:8" ht="15" customHeight="1">
       <c r="H168" s="10"/>
     </row>
-    <row r="169" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="8:8" ht="15" customHeight="1">
       <c r="H169" s="10"/>
     </row>
-    <row r="170" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="8:8" ht="15" customHeight="1">
       <c r="H170" s="10"/>
     </row>
-    <row r="171" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="8:8" ht="15" customHeight="1">
       <c r="H171" s="10"/>
     </row>
-    <row r="172" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="8:8" ht="15" customHeight="1">
       <c r="H172" s="10"/>
     </row>
-    <row r="173" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="8:8" ht="15" customHeight="1">
       <c r="H173" s="10"/>
     </row>
-    <row r="174" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="8:8" ht="15" customHeight="1">
       <c r="H174" s="10"/>
     </row>
-    <row r="175" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="8:8" ht="15" customHeight="1">
       <c r="H175" s="10"/>
     </row>
-    <row r="176" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="8:8" ht="15" customHeight="1">
       <c r="H176" s="10"/>
     </row>
-    <row r="177" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="8:8" ht="15" customHeight="1">
       <c r="H177" s="10"/>
     </row>
-    <row r="178" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="8:8" ht="15" customHeight="1">
       <c r="H178" s="10"/>
     </row>
-    <row r="179" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="8:8" ht="15" customHeight="1">
       <c r="H179" s="10"/>
     </row>
-    <row r="180" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="8:8" ht="15" customHeight="1">
       <c r="H180" s="10"/>
     </row>
-    <row r="181" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="8:8" ht="15" customHeight="1">
       <c r="H181" s="10"/>
     </row>
-    <row r="182" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="8:8" ht="15" customHeight="1">
       <c r="H182" s="10"/>
     </row>
-    <row r="183" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="8:8" ht="15" customHeight="1">
       <c r="H183" s="10"/>
     </row>
-    <row r="184" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="8:8" ht="15" customHeight="1">
       <c r="H184" s="10"/>
     </row>
-    <row r="185" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="8:8" ht="15" customHeight="1">
       <c r="H185" s="10"/>
     </row>
-    <row r="186" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="8:8" ht="15" customHeight="1">
       <c r="H186" s="10"/>
     </row>
-    <row r="187" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="8:8" ht="15" customHeight="1">
       <c r="H187" s="10"/>
     </row>
-    <row r="188" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="8:8" ht="15" customHeight="1">
       <c r="H188" s="10"/>
     </row>
-    <row r="189" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="8:8" ht="15" customHeight="1">
       <c r="H189" s="10"/>
     </row>
-    <row r="190" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="8:8" ht="15" customHeight="1">
       <c r="H190" s="10"/>
     </row>
-    <row r="191" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="8:8" ht="15" customHeight="1">
       <c r="H191" s="10"/>
     </row>
-    <row r="192" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="8:8" ht="15" customHeight="1">
       <c r="H192" s="10"/>
     </row>
-    <row r="193" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="8:8" ht="15" customHeight="1">
       <c r="H193" s="10"/>
     </row>
-    <row r="194" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="8:8" ht="15" customHeight="1">
       <c r="H194" s="10"/>
     </row>
-    <row r="195" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="8:8" ht="15" customHeight="1">
       <c r="H195" s="10"/>
     </row>
-    <row r="196" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="8:8" ht="15" customHeight="1">
       <c r="H196" s="10"/>
     </row>
-    <row r="197" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="8:8" ht="15" customHeight="1">
       <c r="H197" s="10"/>
     </row>
-    <row r="198" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="8:8" ht="15" customHeight="1">
       <c r="H198" s="10"/>
     </row>
-    <row r="199" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="8:8" ht="15" customHeight="1">
       <c r="H199" s="10"/>
     </row>
-    <row r="200" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="8:8" ht="15" customHeight="1">
       <c r="H200" s="10"/>
     </row>
-    <row r="201" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="8:8" ht="15" customHeight="1">
       <c r="H201" s="10"/>
     </row>
-    <row r="202" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="8:8" ht="15" customHeight="1">
       <c r="H202" s="10"/>
     </row>
-    <row r="203" spans="8:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="8:8" ht="15" customHeight="1">
       <c r="H203" s="10"/>
     </row>
   </sheetData>
@@ -4937,14 +4937,14 @@
     <tabColor rgb="FF548235"/>
   </sheetPr>
   <dimension ref="A1:E200"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="13.28515625" customWidth="1"/>
-    <col min="2" max="6" width="12.28515625" customWidth="1"/>
+    <col min="1" max="1" width="13.26953125" customWidth="1"/>
+    <col min="2" max="6" width="12.26953125" customWidth="1"/>
     <col min="7" max="18" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:5" ht="15" customHeight="1">
       <c r="A1" s="18" t="s">
         <v>341</v>
       </c>
@@ -4952,8 +4952,8 @@
       <c r="C1" s="19"/>
       <c r="D1" s="19"/>
     </row>
-    <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="15" customHeight="1"/>
+    <row r="3" spans="1:5" ht="15" customHeight="1">
       <c r="A3" s="11" t="s">
         <v>342</v>
       </c>
@@ -4961,7 +4961,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="15" customHeight="1">
       <c r="A4" s="11" t="s">
         <v>343</v>
       </c>
@@ -4969,7 +4969,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="15" customHeight="1">
       <c r="A5" s="11" t="s">
         <v>344</v>
       </c>
@@ -4977,7 +4977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="15" customHeight="1">
       <c r="A6" s="20" t="s">
         <v>345</v>
       </c>
@@ -4985,7 +4985,7 @@
       <c r="C6" s="19"/>
       <c r="D6" s="19"/>
     </row>
-    <row r="7" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="15" customHeight="1">
       <c r="A7" s="13" t="s">
         <v>346</v>
       </c>
@@ -4999,7 +4999,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="15" customHeight="1">
       <c r="A8" s="6" t="s">
         <v>350</v>
       </c>
@@ -5013,7 +5013,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="15" customHeight="1">
       <c r="A9" s="6" t="s">
         <v>351</v>
       </c>
@@ -5027,7 +5027,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" ht="15" customHeight="1">
       <c r="A10" s="6" t="s">
         <v>352</v>
       </c>
@@ -5041,7 +5041,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" ht="15" customHeight="1">
       <c r="A11" s="14" t="s">
         <v>353</v>
       </c>
@@ -5055,8 +5055,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" ht="15" customHeight="1"/>
+    <row r="13" spans="1:5" ht="15" customHeight="1">
       <c r="A13" s="20" t="s">
         <v>354</v>
       </c>
@@ -5065,7 +5065,7 @@
       <c r="D13" s="19"/>
       <c r="E13" s="19"/>
     </row>
-    <row r="14" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" ht="15" customHeight="1">
       <c r="A14" s="13" t="s">
         <v>355</v>
       </c>
@@ -5082,7 +5082,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" ht="15" customHeight="1">
       <c r="A15" s="6" t="s">
         <v>360</v>
       </c>
@@ -5099,7 +5099,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" ht="15" customHeight="1">
       <c r="A16" s="6" t="s">
         <v>361</v>
       </c>
@@ -5116,7 +5116,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" ht="15" customHeight="1">
       <c r="A17" s="6" t="s">
         <v>362</v>
       </c>
@@ -5133,7 +5133,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" ht="15" customHeight="1">
       <c r="A18" s="6" t="s">
         <v>363</v>
       </c>
@@ -5150,7 +5150,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" ht="15" customHeight="1">
       <c r="A19" s="6" t="s">
         <v>364</v>
       </c>
@@ -5167,7 +5167,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" ht="15" customHeight="1">
       <c r="A20" s="6" t="s">
         <v>365</v>
       </c>
@@ -5184,7 +5184,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" ht="15" customHeight="1">
       <c r="A21" s="6" t="s">
         <v>366</v>
       </c>
@@ -5201,7 +5201,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" ht="15" customHeight="1">
       <c r="A22" s="6" t="s">
         <v>367</v>
       </c>
@@ -5218,7 +5218,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" ht="15" customHeight="1">
       <c r="A23" s="14" t="s">
         <v>368</v>
       </c>
@@ -5235,183 +5235,183 @@
         <v>71</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="49" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="51" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="52" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="53" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="54" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="55" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="56" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="57" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="58" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="59" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="60" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="61" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="62" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="63" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="64" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="65" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="66" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="67" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="68" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="69" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="70" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="71" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="72" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="73" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="74" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="75" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="76" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="77" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="78" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="79" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="80" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="81" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="82" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="83" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="84" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="85" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="86" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="87" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="88" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="89" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="90" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="91" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="92" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="93" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="94" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="95" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="96" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="97" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="98" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="99" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="100" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="101" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="102" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="103" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="104" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="105" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="106" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="107" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="108" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="109" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="110" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="111" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="112" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="113" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="114" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="115" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="116" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="117" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="118" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="119" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="120" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="121" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="122" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="123" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="124" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="125" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="126" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="127" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="128" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="129" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="130" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="131" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="132" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="133" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="134" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="135" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="136" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="137" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="138" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="139" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="140" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="141" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="142" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="143" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="144" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="145" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="146" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="147" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="148" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="149" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="150" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="151" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="152" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="153" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="154" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="155" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="156" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="157" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="158" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="159" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="160" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="161" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="162" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="163" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="164" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="165" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="166" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="167" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="168" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="169" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="170" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="171" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="172" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="173" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="174" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="175" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="176" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="177" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="178" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="179" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="180" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="181" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="182" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="183" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="184" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="185" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="186" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="187" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="188" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="189" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="190" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="191" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="192" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="193" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="194" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="195" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="196" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="197" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="198" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="199" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="200" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:5" ht="15" customHeight="1"/>
+    <row r="25" spans="1:5" ht="15" customHeight="1"/>
+    <row r="26" spans="1:5" ht="15" customHeight="1"/>
+    <row r="27" spans="1:5" ht="15" customHeight="1"/>
+    <row r="28" spans="1:5" ht="15" customHeight="1"/>
+    <row r="29" spans="1:5" ht="15" customHeight="1"/>
+    <row r="30" spans="1:5" ht="15" customHeight="1"/>
+    <row r="31" spans="1:5" ht="15" customHeight="1"/>
+    <row r="32" spans="1:5" ht="15" customHeight="1"/>
+    <row r="33" ht="15" customHeight="1"/>
+    <row r="34" ht="15" customHeight="1"/>
+    <row r="35" ht="15" customHeight="1"/>
+    <row r="36" ht="15" customHeight="1"/>
+    <row r="37" ht="15" customHeight="1"/>
+    <row r="38" ht="15" customHeight="1"/>
+    <row r="39" ht="15" customHeight="1"/>
+    <row r="40" ht="15" customHeight="1"/>
+    <row r="41" ht="15" customHeight="1"/>
+    <row r="42" ht="15" customHeight="1"/>
+    <row r="43" ht="15" customHeight="1"/>
+    <row r="44" ht="15" customHeight="1"/>
+    <row r="45" ht="15" customHeight="1"/>
+    <row r="46" ht="15" customHeight="1"/>
+    <row r="47" ht="15" customHeight="1"/>
+    <row r="48" ht="15" customHeight="1"/>
+    <row r="49" ht="15" customHeight="1"/>
+    <row r="50" ht="15" customHeight="1"/>
+    <row r="51" ht="15" customHeight="1"/>
+    <row r="52" ht="15" customHeight="1"/>
+    <row r="53" ht="15" customHeight="1"/>
+    <row r="54" ht="15" customHeight="1"/>
+    <row r="55" ht="15" customHeight="1"/>
+    <row r="56" ht="15" customHeight="1"/>
+    <row r="57" ht="15" customHeight="1"/>
+    <row r="58" ht="15" customHeight="1"/>
+    <row r="59" ht="15" customHeight="1"/>
+    <row r="60" ht="15" customHeight="1"/>
+    <row r="61" ht="15" customHeight="1"/>
+    <row r="62" ht="15" customHeight="1"/>
+    <row r="63" ht="15" customHeight="1"/>
+    <row r="64" ht="15" customHeight="1"/>
+    <row r="65" ht="15" customHeight="1"/>
+    <row r="66" ht="15" customHeight="1"/>
+    <row r="67" ht="15" customHeight="1"/>
+    <row r="68" ht="15" customHeight="1"/>
+    <row r="69" ht="15" customHeight="1"/>
+    <row r="70" ht="15" customHeight="1"/>
+    <row r="71" ht="15" customHeight="1"/>
+    <row r="72" ht="15" customHeight="1"/>
+    <row r="73" ht="15" customHeight="1"/>
+    <row r="74" ht="15" customHeight="1"/>
+    <row r="75" ht="15" customHeight="1"/>
+    <row r="76" ht="15" customHeight="1"/>
+    <row r="77" ht="15" customHeight="1"/>
+    <row r="78" ht="15" customHeight="1"/>
+    <row r="79" ht="15" customHeight="1"/>
+    <row r="80" ht="15" customHeight="1"/>
+    <row r="81" ht="15" customHeight="1"/>
+    <row r="82" ht="15" customHeight="1"/>
+    <row r="83" ht="15" customHeight="1"/>
+    <row r="84" ht="15" customHeight="1"/>
+    <row r="85" ht="15" customHeight="1"/>
+    <row r="86" ht="15" customHeight="1"/>
+    <row r="87" ht="15" customHeight="1"/>
+    <row r="88" ht="15" customHeight="1"/>
+    <row r="89" ht="15" customHeight="1"/>
+    <row r="90" ht="15" customHeight="1"/>
+    <row r="91" ht="15" customHeight="1"/>
+    <row r="92" ht="15" customHeight="1"/>
+    <row r="93" ht="15" customHeight="1"/>
+    <row r="94" ht="15" customHeight="1"/>
+    <row r="95" ht="15" customHeight="1"/>
+    <row r="96" ht="15" customHeight="1"/>
+    <row r="97" ht="15" customHeight="1"/>
+    <row r="98" ht="15" customHeight="1"/>
+    <row r="99" ht="15" customHeight="1"/>
+    <row r="100" ht="15" customHeight="1"/>
+    <row r="101" ht="15" customHeight="1"/>
+    <row r="102" ht="15" customHeight="1"/>
+    <row r="103" ht="15" customHeight="1"/>
+    <row r="104" ht="15" customHeight="1"/>
+    <row r="105" ht="15" customHeight="1"/>
+    <row r="106" ht="15" customHeight="1"/>
+    <row r="107" ht="15" customHeight="1"/>
+    <row r="108" ht="15" customHeight="1"/>
+    <row r="109" ht="15" customHeight="1"/>
+    <row r="110" ht="15" customHeight="1"/>
+    <row r="111" ht="15" customHeight="1"/>
+    <row r="112" ht="15" customHeight="1"/>
+    <row r="113" ht="15" customHeight="1"/>
+    <row r="114" ht="15" customHeight="1"/>
+    <row r="115" ht="15" customHeight="1"/>
+    <row r="116" ht="15" customHeight="1"/>
+    <row r="117" ht="15" customHeight="1"/>
+    <row r="118" ht="15" customHeight="1"/>
+    <row r="119" ht="15" customHeight="1"/>
+    <row r="120" ht="15" customHeight="1"/>
+    <row r="121" ht="15" customHeight="1"/>
+    <row r="122" ht="15" customHeight="1"/>
+    <row r="123" ht="15" customHeight="1"/>
+    <row r="124" ht="15" customHeight="1"/>
+    <row r="125" ht="15" customHeight="1"/>
+    <row r="126" ht="15" customHeight="1"/>
+    <row r="127" ht="15" customHeight="1"/>
+    <row r="128" ht="15" customHeight="1"/>
+    <row r="129" ht="15" customHeight="1"/>
+    <row r="130" ht="15" customHeight="1"/>
+    <row r="131" ht="15" customHeight="1"/>
+    <row r="132" ht="15" customHeight="1"/>
+    <row r="133" ht="15" customHeight="1"/>
+    <row r="134" ht="15" customHeight="1"/>
+    <row r="135" ht="15" customHeight="1"/>
+    <row r="136" ht="15" customHeight="1"/>
+    <row r="137" ht="15" customHeight="1"/>
+    <row r="138" ht="15" customHeight="1"/>
+    <row r="139" ht="15" customHeight="1"/>
+    <row r="140" ht="15" customHeight="1"/>
+    <row r="141" ht="15" customHeight="1"/>
+    <row r="142" ht="15" customHeight="1"/>
+    <row r="143" ht="15" customHeight="1"/>
+    <row r="144" ht="15" customHeight="1"/>
+    <row r="145" ht="15" customHeight="1"/>
+    <row r="146" ht="15" customHeight="1"/>
+    <row r="147" ht="15" customHeight="1"/>
+    <row r="148" ht="15" customHeight="1"/>
+    <row r="149" ht="15" customHeight="1"/>
+    <row r="150" ht="15" customHeight="1"/>
+    <row r="151" ht="15" customHeight="1"/>
+    <row r="152" ht="15" customHeight="1"/>
+    <row r="153" ht="15" customHeight="1"/>
+    <row r="154" ht="15" customHeight="1"/>
+    <row r="155" ht="15" customHeight="1"/>
+    <row r="156" ht="15" customHeight="1"/>
+    <row r="157" ht="15" customHeight="1"/>
+    <row r="158" ht="15" customHeight="1"/>
+    <row r="159" ht="15" customHeight="1"/>
+    <row r="160" ht="15" customHeight="1"/>
+    <row r="161" ht="15" customHeight="1"/>
+    <row r="162" ht="15" customHeight="1"/>
+    <row r="163" ht="15" customHeight="1"/>
+    <row r="164" ht="15" customHeight="1"/>
+    <row r="165" ht="15" customHeight="1"/>
+    <row r="166" ht="15" customHeight="1"/>
+    <row r="167" ht="15" customHeight="1"/>
+    <row r="168" ht="15" customHeight="1"/>
+    <row r="169" ht="15" customHeight="1"/>
+    <row r="170" ht="15" customHeight="1"/>
+    <row r="171" ht="15" customHeight="1"/>
+    <row r="172" ht="15" customHeight="1"/>
+    <row r="173" ht="15" customHeight="1"/>
+    <row r="174" ht="15" customHeight="1"/>
+    <row r="175" ht="15" customHeight="1"/>
+    <row r="176" ht="15" customHeight="1"/>
+    <row r="177" ht="15" customHeight="1"/>
+    <row r="178" ht="15" customHeight="1"/>
+    <row r="179" ht="15" customHeight="1"/>
+    <row r="180" ht="15" customHeight="1"/>
+    <row r="181" ht="15" customHeight="1"/>
+    <row r="182" ht="15" customHeight="1"/>
+    <row r="183" ht="15" customHeight="1"/>
+    <row r="184" ht="15" customHeight="1"/>
+    <row r="185" ht="15" customHeight="1"/>
+    <row r="186" ht="15" customHeight="1"/>
+    <row r="187" ht="15" customHeight="1"/>
+    <row r="188" ht="15" customHeight="1"/>
+    <row r="189" ht="15" customHeight="1"/>
+    <row r="190" ht="15" customHeight="1"/>
+    <row r="191" ht="15" customHeight="1"/>
+    <row r="192" ht="15" customHeight="1"/>
+    <row r="193" ht="15" customHeight="1"/>
+    <row r="194" ht="15" customHeight="1"/>
+    <row r="195" ht="15" customHeight="1"/>
+    <row r="196" ht="15" customHeight="1"/>
+    <row r="197" ht="15" customHeight="1"/>
+    <row r="198" ht="15" customHeight="1"/>
+    <row r="199" ht="15" customHeight="1"/>
+    <row r="200" ht="15" customHeight="1"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
@@ -5428,250 +5428,250 @@
     <tabColor rgb="FF808080"/>
   </sheetPr>
   <dimension ref="A1:A200"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="99.28515625" customWidth="1"/>
+    <col min="1" max="1" width="99.26953125" customWidth="1"/>
     <col min="2" max="18" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="15" customHeight="1">
       <c r="A1" s="15" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" ht="15" customHeight="1">
       <c r="A2" s="16"/>
     </row>
-    <row r="3" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" ht="15" customHeight="1">
       <c r="A3" s="16" t="s">
         <v>370</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" ht="15" customHeight="1">
       <c r="A4" s="16" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" ht="15" customHeight="1">
       <c r="A5" s="16" t="s">
         <v>372</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" ht="15" customHeight="1">
       <c r="A6" s="16"/>
     </row>
-    <row r="7" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" ht="15" customHeight="1">
       <c r="A7" s="16" t="s">
         <v>373</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" ht="15" customHeight="1">
       <c r="A8" s="16" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" ht="15" customHeight="1">
       <c r="A9" s="16"/>
     </row>
-    <row r="10" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" ht="15" customHeight="1">
       <c r="A10" s="16" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" ht="15" customHeight="1">
       <c r="A11" s="16" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="18" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="19" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="49" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="51" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="52" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="53" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="54" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="55" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="56" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="57" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="58" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="59" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="60" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="61" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="62" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="63" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="64" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="65" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="66" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="67" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="68" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="69" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="70" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="71" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="72" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="73" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="74" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="75" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="76" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="77" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="78" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="79" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="80" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="81" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="82" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="83" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="84" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="85" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="86" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="87" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="88" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="89" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="90" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="91" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="92" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="93" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="94" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="95" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="96" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="97" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="98" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="99" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="100" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="101" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="102" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="103" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="104" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="105" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="106" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="107" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="108" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="109" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="110" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="111" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="112" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="113" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="114" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="115" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="116" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="117" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="118" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="119" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="120" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="121" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="122" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="123" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="124" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="125" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="126" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="127" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="128" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="129" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="130" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="131" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="132" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="133" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="134" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="135" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="136" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="137" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="138" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="139" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="140" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="141" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="142" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="143" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="144" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="145" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="146" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="147" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="148" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="149" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="150" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="151" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="152" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="153" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="154" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="155" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="156" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="157" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="158" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="159" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="160" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="161" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="162" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="163" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="164" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="165" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="166" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="167" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="168" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="169" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="170" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="171" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="172" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="173" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="174" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="175" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="176" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="177" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="178" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="179" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="180" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="181" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="182" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="183" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="184" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="185" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="186" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="187" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="188" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="189" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="190" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="191" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="192" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="193" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="194" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="195" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="196" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="197" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="198" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="199" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="200" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:1" ht="15" customHeight="1"/>
+    <row r="13" spans="1:1" ht="15" customHeight="1"/>
+    <row r="14" spans="1:1" ht="15" customHeight="1"/>
+    <row r="15" spans="1:1" ht="15" customHeight="1"/>
+    <row r="16" spans="1:1" ht="15" customHeight="1"/>
+    <row r="17" ht="15" customHeight="1"/>
+    <row r="18" ht="15" customHeight="1"/>
+    <row r="19" ht="15" customHeight="1"/>
+    <row r="20" ht="15" customHeight="1"/>
+    <row r="21" ht="15" customHeight="1"/>
+    <row r="22" ht="15" customHeight="1"/>
+    <row r="23" ht="15" customHeight="1"/>
+    <row r="24" ht="15" customHeight="1"/>
+    <row r="25" ht="15" customHeight="1"/>
+    <row r="26" ht="15" customHeight="1"/>
+    <row r="27" ht="15" customHeight="1"/>
+    <row r="28" ht="15" customHeight="1"/>
+    <row r="29" ht="15" customHeight="1"/>
+    <row r="30" ht="15" customHeight="1"/>
+    <row r="31" ht="15" customHeight="1"/>
+    <row r="32" ht="15" customHeight="1"/>
+    <row r="33" ht="15" customHeight="1"/>
+    <row r="34" ht="15" customHeight="1"/>
+    <row r="35" ht="15" customHeight="1"/>
+    <row r="36" ht="15" customHeight="1"/>
+    <row r="37" ht="15" customHeight="1"/>
+    <row r="38" ht="15" customHeight="1"/>
+    <row r="39" ht="15" customHeight="1"/>
+    <row r="40" ht="15" customHeight="1"/>
+    <row r="41" ht="15" customHeight="1"/>
+    <row r="42" ht="15" customHeight="1"/>
+    <row r="43" ht="15" customHeight="1"/>
+    <row r="44" ht="15" customHeight="1"/>
+    <row r="45" ht="15" customHeight="1"/>
+    <row r="46" ht="15" customHeight="1"/>
+    <row r="47" ht="15" customHeight="1"/>
+    <row r="48" ht="15" customHeight="1"/>
+    <row r="49" ht="15" customHeight="1"/>
+    <row r="50" ht="15" customHeight="1"/>
+    <row r="51" ht="15" customHeight="1"/>
+    <row r="52" ht="15" customHeight="1"/>
+    <row r="53" ht="15" customHeight="1"/>
+    <row r="54" ht="15" customHeight="1"/>
+    <row r="55" ht="15" customHeight="1"/>
+    <row r="56" ht="15" customHeight="1"/>
+    <row r="57" ht="15" customHeight="1"/>
+    <row r="58" ht="15" customHeight="1"/>
+    <row r="59" ht="15" customHeight="1"/>
+    <row r="60" ht="15" customHeight="1"/>
+    <row r="61" ht="15" customHeight="1"/>
+    <row r="62" ht="15" customHeight="1"/>
+    <row r="63" ht="15" customHeight="1"/>
+    <row r="64" ht="15" customHeight="1"/>
+    <row r="65" ht="15" customHeight="1"/>
+    <row r="66" ht="15" customHeight="1"/>
+    <row r="67" ht="15" customHeight="1"/>
+    <row r="68" ht="15" customHeight="1"/>
+    <row r="69" ht="15" customHeight="1"/>
+    <row r="70" ht="15" customHeight="1"/>
+    <row r="71" ht="15" customHeight="1"/>
+    <row r="72" ht="15" customHeight="1"/>
+    <row r="73" ht="15" customHeight="1"/>
+    <row r="74" ht="15" customHeight="1"/>
+    <row r="75" ht="15" customHeight="1"/>
+    <row r="76" ht="15" customHeight="1"/>
+    <row r="77" ht="15" customHeight="1"/>
+    <row r="78" ht="15" customHeight="1"/>
+    <row r="79" ht="15" customHeight="1"/>
+    <row r="80" ht="15" customHeight="1"/>
+    <row r="81" ht="15" customHeight="1"/>
+    <row r="82" ht="15" customHeight="1"/>
+    <row r="83" ht="15" customHeight="1"/>
+    <row r="84" ht="15" customHeight="1"/>
+    <row r="85" ht="15" customHeight="1"/>
+    <row r="86" ht="15" customHeight="1"/>
+    <row r="87" ht="15" customHeight="1"/>
+    <row r="88" ht="15" customHeight="1"/>
+    <row r="89" ht="15" customHeight="1"/>
+    <row r="90" ht="15" customHeight="1"/>
+    <row r="91" ht="15" customHeight="1"/>
+    <row r="92" ht="15" customHeight="1"/>
+    <row r="93" ht="15" customHeight="1"/>
+    <row r="94" ht="15" customHeight="1"/>
+    <row r="95" ht="15" customHeight="1"/>
+    <row r="96" ht="15" customHeight="1"/>
+    <row r="97" ht="15" customHeight="1"/>
+    <row r="98" ht="15" customHeight="1"/>
+    <row r="99" ht="15" customHeight="1"/>
+    <row r="100" ht="15" customHeight="1"/>
+    <row r="101" ht="15" customHeight="1"/>
+    <row r="102" ht="15" customHeight="1"/>
+    <row r="103" ht="15" customHeight="1"/>
+    <row r="104" ht="15" customHeight="1"/>
+    <row r="105" ht="15" customHeight="1"/>
+    <row r="106" ht="15" customHeight="1"/>
+    <row r="107" ht="15" customHeight="1"/>
+    <row r="108" ht="15" customHeight="1"/>
+    <row r="109" ht="15" customHeight="1"/>
+    <row r="110" ht="15" customHeight="1"/>
+    <row r="111" ht="15" customHeight="1"/>
+    <row r="112" ht="15" customHeight="1"/>
+    <row r="113" ht="15" customHeight="1"/>
+    <row r="114" ht="15" customHeight="1"/>
+    <row r="115" ht="15" customHeight="1"/>
+    <row r="116" ht="15" customHeight="1"/>
+    <row r="117" ht="15" customHeight="1"/>
+    <row r="118" ht="15" customHeight="1"/>
+    <row r="119" ht="15" customHeight="1"/>
+    <row r="120" ht="15" customHeight="1"/>
+    <row r="121" ht="15" customHeight="1"/>
+    <row r="122" ht="15" customHeight="1"/>
+    <row r="123" ht="15" customHeight="1"/>
+    <row r="124" ht="15" customHeight="1"/>
+    <row r="125" ht="15" customHeight="1"/>
+    <row r="126" ht="15" customHeight="1"/>
+    <row r="127" ht="15" customHeight="1"/>
+    <row r="128" ht="15" customHeight="1"/>
+    <row r="129" ht="15" customHeight="1"/>
+    <row r="130" ht="15" customHeight="1"/>
+    <row r="131" ht="15" customHeight="1"/>
+    <row r="132" ht="15" customHeight="1"/>
+    <row r="133" ht="15" customHeight="1"/>
+    <row r="134" ht="15" customHeight="1"/>
+    <row r="135" ht="15" customHeight="1"/>
+    <row r="136" ht="15" customHeight="1"/>
+    <row r="137" ht="15" customHeight="1"/>
+    <row r="138" ht="15" customHeight="1"/>
+    <row r="139" ht="15" customHeight="1"/>
+    <row r="140" ht="15" customHeight="1"/>
+    <row r="141" ht="15" customHeight="1"/>
+    <row r="142" ht="15" customHeight="1"/>
+    <row r="143" ht="15" customHeight="1"/>
+    <row r="144" ht="15" customHeight="1"/>
+    <row r="145" ht="15" customHeight="1"/>
+    <row r="146" ht="15" customHeight="1"/>
+    <row r="147" ht="15" customHeight="1"/>
+    <row r="148" ht="15" customHeight="1"/>
+    <row r="149" ht="15" customHeight="1"/>
+    <row r="150" ht="15" customHeight="1"/>
+    <row r="151" ht="15" customHeight="1"/>
+    <row r="152" ht="15" customHeight="1"/>
+    <row r="153" ht="15" customHeight="1"/>
+    <row r="154" ht="15" customHeight="1"/>
+    <row r="155" ht="15" customHeight="1"/>
+    <row r="156" ht="15" customHeight="1"/>
+    <row r="157" ht="15" customHeight="1"/>
+    <row r="158" ht="15" customHeight="1"/>
+    <row r="159" ht="15" customHeight="1"/>
+    <row r="160" ht="15" customHeight="1"/>
+    <row r="161" ht="15" customHeight="1"/>
+    <row r="162" ht="15" customHeight="1"/>
+    <row r="163" ht="15" customHeight="1"/>
+    <row r="164" ht="15" customHeight="1"/>
+    <row r="165" ht="15" customHeight="1"/>
+    <row r="166" ht="15" customHeight="1"/>
+    <row r="167" ht="15" customHeight="1"/>
+    <row r="168" ht="15" customHeight="1"/>
+    <row r="169" ht="15" customHeight="1"/>
+    <row r="170" ht="15" customHeight="1"/>
+    <row r="171" ht="15" customHeight="1"/>
+    <row r="172" ht="15" customHeight="1"/>
+    <row r="173" ht="15" customHeight="1"/>
+    <row r="174" ht="15" customHeight="1"/>
+    <row r="175" ht="15" customHeight="1"/>
+    <row r="176" ht="15" customHeight="1"/>
+    <row r="177" ht="15" customHeight="1"/>
+    <row r="178" ht="15" customHeight="1"/>
+    <row r="179" ht="15" customHeight="1"/>
+    <row r="180" ht="15" customHeight="1"/>
+    <row r="181" ht="15" customHeight="1"/>
+    <row r="182" ht="15" customHeight="1"/>
+    <row r="183" ht="15" customHeight="1"/>
+    <row r="184" ht="15" customHeight="1"/>
+    <row r="185" ht="15" customHeight="1"/>
+    <row r="186" ht="15" customHeight="1"/>
+    <row r="187" ht="15" customHeight="1"/>
+    <row r="188" ht="15" customHeight="1"/>
+    <row r="189" ht="15" customHeight="1"/>
+    <row r="190" ht="15" customHeight="1"/>
+    <row r="191" ht="15" customHeight="1"/>
+    <row r="192" ht="15" customHeight="1"/>
+    <row r="193" ht="15" customHeight="1"/>
+    <row r="194" ht="15" customHeight="1"/>
+    <row r="195" ht="15" customHeight="1"/>
+    <row r="196" ht="15" customHeight="1"/>
+    <row r="197" ht="15" customHeight="1"/>
+    <row r="198" ht="15" customHeight="1"/>
+    <row r="199" ht="15" customHeight="1"/>
+    <row r="200" ht="15" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
release: ship Alpha v2.6.0-hotfix.1
</commit_message>
<xml_diff>
--- a/assets/source-archive/alpha-v260-xlsx-import/sources/法术卡列表.xlsx
+++ b/assets/source-archive/alpha-v260-xlsx-import/sources/法术卡列表.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Project\WizardCard-Design\Alpha 现有卡池\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7315636F-2767-411D-B26A-D7370BCCA7D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D625B10B-8B98-4AAB-A63A-306C67F5A51B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4958,7 +4958,7 @@
         <v>342</v>
       </c>
       <c r="B3" s="12">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="15" customHeight="1">
@@ -4966,7 +4966,7 @@
         <v>343</v>
       </c>
       <c r="B4" s="12">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15" customHeight="1">
@@ -5046,10 +5046,10 @@
         <v>353</v>
       </c>
       <c r="B11" s="14">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C11" s="14">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D11" s="14">
         <v>0</v>
@@ -5232,7 +5232,7 @@
         <v>17</v>
       </c>
       <c r="E23" s="14">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="15" customHeight="1"/>

</xml_diff>